<commit_message>
Paneles instalados por inversor (cantidad y potencia en Wp)
- Migracion 011: inversores.cantidad_paneles y potencia_panel_wp.
- API, formulario, listado y detalle del inversor; carga masiva.
- Total de grupo y proyecto suma inversores; lotes solo si no hay detalle.
- Pruebas y documentacion.
</commit_message>
<xml_diff>
--- a/database/seeds/plantilla_carga_masiva.xlsx
+++ b/database/seeds/plantilla_carga_masiva.xlsx
@@ -302,12 +302,26 @@
         </r>
       </text>
     </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <t>Paneles instalados en el inversor (con la potencia por panel).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
+          <t>Vatios pico de cada panel, por ejemplo 550.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="74">
   <si>
     <t>PLANTILLA DE CARGA MASIVA — CLIENTES, PROYECTOS, GRUPOS E INVERSORES</t>
   </si>
@@ -508,6 +522,12 @@
   </si>
   <si>
     <t>Estado</t>
+  </si>
+  <si>
+    <t>Cantidad de paneles</t>
+  </si>
+  <si>
+    <t>Potencia por panel (Wp)</t>
   </si>
   <si>
     <t>Huawei</t>
@@ -5329,7 +5349,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J501"/>
+  <dimension ref="A1:L501"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -5341,9 +5361,11 @@
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>37</v>
       </c>
@@ -5374,8 +5396,14 @@
       <c r="J1" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="K1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>46</v>
       </c>
@@ -5383,16 +5411,16 @@
         <v>58</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>1</v>
@@ -5401,1507 +5429,1513 @@
         <v>100</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="3">
+        <v>182</v>
+      </c>
+      <c r="L2" s="3">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F17" s="5"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F19" s="5"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F21" s="5"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F22" s="5"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F24" s="5"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F25" s="5"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F26" s="5"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F27" s="5"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F28" s="5"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F29" s="5"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F30" s="5"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F31" s="5"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F32" s="5"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F33" s="5"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F34" s="5"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F35" s="5"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F36" s="5"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F37" s="5"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F38" s="5"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F39" s="5"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F40" s="5"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F41" s="5"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F42" s="5"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F43" s="5"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F44" s="5"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F45" s="5"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F46" s="5"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F47" s="5"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F48" s="5"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F49" s="5"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F50" s="5"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F51" s="5"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F52" s="5"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F53" s="5"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F54" s="5"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F55" s="5"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F56" s="5"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F57" s="5"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F58" s="5"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F59" s="5"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F60" s="5"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F61" s="5"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F62" s="5"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F63" s="5"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F64" s="5"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F65" s="5"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F66" s="5"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F67" s="5"/>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F68" s="5"/>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F69" s="5"/>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F70" s="5"/>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F71" s="5"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F72" s="5"/>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F73" s="5"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F74" s="5"/>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F75" s="5"/>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F76" s="5"/>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F77" s="5"/>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F78" s="5"/>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F79" s="5"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F80" s="5"/>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F81" s="5"/>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F82" s="5"/>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F83" s="5"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F84" s="5"/>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F85" s="5"/>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F86" s="5"/>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F87" s="5"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F88" s="5"/>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F89" s="5"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F90" s="5"/>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F91" s="5"/>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F92" s="5"/>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F93" s="5"/>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F94" s="5"/>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F95" s="5"/>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F96" s="5"/>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F97" s="5"/>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F98" s="5"/>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F99" s="5"/>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F100" s="5"/>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F101" s="5"/>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F102" s="5"/>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F103" s="5"/>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F104" s="5"/>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F105" s="5"/>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F106" s="5"/>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F107" s="5"/>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F108" s="5"/>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F109" s="5"/>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F110" s="5"/>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F111" s="5"/>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F112" s="5"/>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F113" s="5"/>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F114" s="5"/>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F115" s="5"/>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F116" s="5"/>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F117" s="5"/>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F118" s="5"/>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F119" s="5"/>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F120" s="5"/>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F121" s="5"/>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F122" s="5"/>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F123" s="5"/>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F124" s="5"/>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F125" s="5"/>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F126" s="5"/>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F127" s="5"/>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F128" s="5"/>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F129" s="5"/>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F130" s="5"/>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F131" s="5"/>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F132" s="5"/>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F133" s="5"/>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F134" s="5"/>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F135" s="5"/>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F136" s="5"/>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F137" s="5"/>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F138" s="5"/>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F139" s="5"/>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F140" s="5"/>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F141" s="5"/>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F142" s="5"/>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F143" s="5"/>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F144" s="5"/>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F145" s="5"/>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F146" s="5"/>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F147" s="5"/>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F148" s="5"/>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F149" s="5"/>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F150" s="5"/>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F151" s="5"/>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F152" s="5"/>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F153" s="5"/>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F154" s="5"/>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F155" s="5"/>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F156" s="5"/>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F157" s="5"/>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F158" s="5"/>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F159" s="5"/>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F160" s="5"/>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F161" s="5"/>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F162" s="5"/>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F163" s="5"/>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F164" s="5"/>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F165" s="5"/>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F166" s="5"/>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F167" s="5"/>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F168" s="5"/>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F169" s="5"/>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F170" s="5"/>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F171" s="5"/>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F172" s="5"/>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F173" s="5"/>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F174" s="5"/>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F175" s="5"/>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F176" s="5"/>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F177" s="5"/>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F178" s="5"/>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F179" s="5"/>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F180" s="5"/>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F181" s="5"/>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F182" s="5"/>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F183" s="5"/>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F184" s="5"/>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F185" s="5"/>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F186" s="5"/>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F187" s="5"/>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F188" s="5"/>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F189" s="5"/>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F190" s="5"/>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F191" s="5"/>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F192" s="5"/>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F193" s="5"/>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F194" s="5"/>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F195" s="5"/>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F196" s="5"/>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F197" s="5"/>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F198" s="5"/>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F199" s="5"/>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F200" s="5"/>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F201" s="5"/>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F202" s="5"/>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F203" s="5"/>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F204" s="5"/>
     </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F205" s="5"/>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F206" s="5"/>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F207" s="5"/>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F208" s="5"/>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F209" s="5"/>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F210" s="5"/>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F211" s="5"/>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F212" s="5"/>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F213" s="5"/>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F214" s="5"/>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F215" s="5"/>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F216" s="5"/>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F217" s="5"/>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F218" s="5"/>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F219" s="5"/>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F220" s="5"/>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F221" s="5"/>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F222" s="5"/>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F223" s="5"/>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F224" s="5"/>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F225" s="5"/>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F226" s="5"/>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F227" s="5"/>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F228" s="5"/>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F229" s="5"/>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F230" s="5"/>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F231" s="5"/>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F232" s="5"/>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F233" s="5"/>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F234" s="5"/>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F235" s="5"/>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F236" s="5"/>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F237" s="5"/>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F238" s="5"/>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F239" s="5"/>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F240" s="5"/>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F241" s="5"/>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F242" s="5"/>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F243" s="5"/>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F244" s="5"/>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F245" s="5"/>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F246" s="5"/>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F247" s="5"/>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F248" s="5"/>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F249" s="5"/>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F250" s="5"/>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F251" s="5"/>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F252" s="5"/>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F253" s="5"/>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F254" s="5"/>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F255" s="5"/>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F256" s="5"/>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F257" s="5"/>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F258" s="5"/>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F259" s="5"/>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F260" s="5"/>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F261" s="5"/>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F262" s="5"/>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F263" s="5"/>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F264" s="5"/>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F265" s="5"/>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F266" s="5"/>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F267" s="5"/>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F268" s="5"/>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F269" s="5"/>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F270" s="5"/>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F271" s="5"/>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F272" s="5"/>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F273" s="5"/>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F274" s="5"/>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F275" s="5"/>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F276" s="5"/>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F277" s="5"/>
     </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F278" s="5"/>
     </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F279" s="5"/>
     </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F280" s="5"/>
     </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F281" s="5"/>
     </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F282" s="5"/>
     </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F283" s="5"/>
     </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F284" s="5"/>
     </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F285" s="5"/>
     </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F286" s="5"/>
     </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F287" s="5"/>
     </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F288" s="5"/>
     </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F289" s="5"/>
     </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F290" s="5"/>
     </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F291" s="5"/>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F292" s="5"/>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F293" s="5"/>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F294" s="5"/>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F295" s="5"/>
     </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F296" s="5"/>
     </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F297" s="5"/>
     </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F298" s="5"/>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F299" s="5"/>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F300" s="5"/>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F301" s="5"/>
     </row>
-    <row r="302" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F302" s="5"/>
     </row>
-    <row r="303" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F303" s="5"/>
     </row>
-    <row r="304" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F304" s="5"/>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F305" s="5"/>
     </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F306" s="5"/>
     </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F307" s="5"/>
     </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F308" s="5"/>
     </row>
-    <row r="309" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F309" s="5"/>
     </row>
-    <row r="310" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F310" s="5"/>
     </row>
-    <row r="311" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F311" s="5"/>
     </row>
-    <row r="312" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F312" s="5"/>
     </row>
-    <row r="313" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F313" s="5"/>
     </row>
-    <row r="314" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F314" s="5"/>
     </row>
-    <row r="315" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F315" s="5"/>
     </row>
-    <row r="316" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F316" s="5"/>
     </row>
-    <row r="317" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F317" s="5"/>
     </row>
-    <row r="318" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F318" s="5"/>
     </row>
-    <row r="319" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F319" s="5"/>
     </row>
-    <row r="320" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F320" s="5"/>
     </row>
-    <row r="321" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F321" s="5"/>
     </row>
-    <row r="322" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F322" s="5"/>
     </row>
-    <row r="323" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F323" s="5"/>
     </row>
-    <row r="324" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F324" s="5"/>
     </row>
-    <row r="325" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F325" s="5"/>
     </row>
-    <row r="326" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F326" s="5"/>
     </row>
-    <row r="327" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F327" s="5"/>
     </row>
-    <row r="328" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F328" s="5"/>
     </row>
-    <row r="329" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F329" s="5"/>
     </row>
-    <row r="330" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F330" s="5"/>
     </row>
-    <row r="331" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F331" s="5"/>
     </row>
-    <row r="332" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F332" s="5"/>
     </row>
-    <row r="333" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F333" s="5"/>
     </row>
-    <row r="334" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F334" s="5"/>
     </row>
-    <row r="335" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F335" s="5"/>
     </row>
-    <row r="336" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F336" s="5"/>
     </row>
-    <row r="337" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F337" s="5"/>
     </row>
-    <row r="338" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F338" s="5"/>
     </row>
-    <row r="339" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F339" s="5"/>
     </row>
-    <row r="340" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F340" s="5"/>
     </row>
-    <row r="341" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F341" s="5"/>
     </row>
-    <row r="342" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F342" s="5"/>
     </row>
-    <row r="343" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F343" s="5"/>
     </row>
-    <row r="344" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F344" s="5"/>
     </row>
-    <row r="345" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F345" s="5"/>
     </row>
-    <row r="346" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F346" s="5"/>
     </row>
-    <row r="347" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F347" s="5"/>
     </row>
-    <row r="348" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F348" s="5"/>
     </row>
-    <row r="349" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F349" s="5"/>
     </row>
-    <row r="350" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F350" s="5"/>
     </row>
-    <row r="351" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F351" s="5"/>
     </row>
-    <row r="352" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F352" s="5"/>
     </row>
-    <row r="353" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F353" s="5"/>
     </row>
-    <row r="354" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F354" s="5"/>
     </row>
-    <row r="355" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F355" s="5"/>
     </row>
-    <row r="356" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F356" s="5"/>
     </row>
-    <row r="357" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F357" s="5"/>
     </row>
-    <row r="358" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F358" s="5"/>
     </row>
-    <row r="359" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F359" s="5"/>
     </row>
-    <row r="360" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F360" s="5"/>
     </row>
-    <row r="361" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F361" s="5"/>
     </row>
-    <row r="362" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F362" s="5"/>
     </row>
-    <row r="363" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F363" s="5"/>
     </row>
-    <row r="364" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F364" s="5"/>
     </row>
-    <row r="365" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F365" s="5"/>
     </row>
-    <row r="366" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F366" s="5"/>
     </row>
-    <row r="367" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F367" s="5"/>
     </row>
-    <row r="368" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F368" s="5"/>
     </row>
-    <row r="369" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F369" s="5"/>
     </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F370" s="5"/>
     </row>
-    <row r="371" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F371" s="5"/>
     </row>
-    <row r="372" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F372" s="5"/>
     </row>
-    <row r="373" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F373" s="5"/>
     </row>
-    <row r="374" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F374" s="5"/>
     </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F375" s="5"/>
     </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F376" s="5"/>
     </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F377" s="5"/>
     </row>
-    <row r="378" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F378" s="5"/>
     </row>
-    <row r="379" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F379" s="5"/>
     </row>
-    <row r="380" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F380" s="5"/>
     </row>
-    <row r="381" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F381" s="5"/>
     </row>
-    <row r="382" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F382" s="5"/>
     </row>
-    <row r="383" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F383" s="5"/>
     </row>
-    <row r="384" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F384" s="5"/>
     </row>
-    <row r="385" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F385" s="5"/>
     </row>
-    <row r="386" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F386" s="5"/>
     </row>
-    <row r="387" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F387" s="5"/>
     </row>
-    <row r="388" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F388" s="5"/>
     </row>
-    <row r="389" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F389" s="5"/>
     </row>
-    <row r="390" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F390" s="5"/>
     </row>
-    <row r="391" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F391" s="5"/>
     </row>
-    <row r="392" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F392" s="5"/>
     </row>
-    <row r="393" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F393" s="5"/>
     </row>
-    <row r="394" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F394" s="5"/>
     </row>
-    <row r="395" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F395" s="5"/>
     </row>
-    <row r="396" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F396" s="5"/>
     </row>
-    <row r="397" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F397" s="5"/>
     </row>
-    <row r="398" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F398" s="5"/>
     </row>
-    <row r="399" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F399" s="5"/>
     </row>
-    <row r="400" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F400" s="5"/>
     </row>
-    <row r="401" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F401" s="5"/>
     </row>
-    <row r="402" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F402" s="5"/>
     </row>
-    <row r="403" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F403" s="5"/>
     </row>
-    <row r="404" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F404" s="5"/>
     </row>
-    <row r="405" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F405" s="5"/>
     </row>
-    <row r="406" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F406" s="5"/>
     </row>
-    <row r="407" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F407" s="5"/>
     </row>
-    <row r="408" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F408" s="5"/>
     </row>
-    <row r="409" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F409" s="5"/>
     </row>
-    <row r="410" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F410" s="5"/>
     </row>
-    <row r="411" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F411" s="5"/>
     </row>
-    <row r="412" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F412" s="5"/>
     </row>
-    <row r="413" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F413" s="5"/>
     </row>
-    <row r="414" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F414" s="5"/>
     </row>
-    <row r="415" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F415" s="5"/>
     </row>
-    <row r="416" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F416" s="5"/>
     </row>
-    <row r="417" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F417" s="5"/>
     </row>
-    <row r="418" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F418" s="5"/>
     </row>
-    <row r="419" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F419" s="5"/>
     </row>
-    <row r="420" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F420" s="5"/>
     </row>
-    <row r="421" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F421" s="5"/>
     </row>
-    <row r="422" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F422" s="5"/>
     </row>
-    <row r="423" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F423" s="5"/>
     </row>
-    <row r="424" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F424" s="5"/>
     </row>
-    <row r="425" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F425" s="5"/>
     </row>
-    <row r="426" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F426" s="5"/>
     </row>
-    <row r="427" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F427" s="5"/>
     </row>
-    <row r="428" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F428" s="5"/>
     </row>
-    <row r="429" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F429" s="5"/>
     </row>
-    <row r="430" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F430" s="5"/>
     </row>
-    <row r="431" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F431" s="5"/>
     </row>
-    <row r="432" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F432" s="5"/>
     </row>
-    <row r="433" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F433" s="5"/>
     </row>
-    <row r="434" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F434" s="5"/>
     </row>
-    <row r="435" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F435" s="5"/>
     </row>
-    <row r="436" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F436" s="5"/>
     </row>
-    <row r="437" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F437" s="5"/>
     </row>
-    <row r="438" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F438" s="5"/>
     </row>
-    <row r="439" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F439" s="5"/>
     </row>
-    <row r="440" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F440" s="5"/>
     </row>
-    <row r="441" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F441" s="5"/>
     </row>
-    <row r="442" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F442" s="5"/>
     </row>
-    <row r="443" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F443" s="5"/>
     </row>
-    <row r="444" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F444" s="5"/>
     </row>
-    <row r="445" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F445" s="5"/>
     </row>
-    <row r="446" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F446" s="5"/>
     </row>
-    <row r="447" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F447" s="5"/>
     </row>
-    <row r="448" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F448" s="5"/>
     </row>
-    <row r="449" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F449" s="5"/>
     </row>
-    <row r="450" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F450" s="5"/>
     </row>
-    <row r="451" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F451" s="5"/>
     </row>
-    <row r="452" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F452" s="5"/>
     </row>
-    <row r="453" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F453" s="5"/>
     </row>
-    <row r="454" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F454" s="5"/>
     </row>
-    <row r="455" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F455" s="5"/>
     </row>
-    <row r="456" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F456" s="5"/>
     </row>
-    <row r="457" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F457" s="5"/>
     </row>
-    <row r="458" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F458" s="5"/>
     </row>
-    <row r="459" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F459" s="5"/>
     </row>
-    <row r="460" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F460" s="5"/>
     </row>
-    <row r="461" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F461" s="5"/>
     </row>
-    <row r="462" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F462" s="5"/>
     </row>
-    <row r="463" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F463" s="5"/>
     </row>
-    <row r="464" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F464" s="5"/>
     </row>
-    <row r="465" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F465" s="5"/>
     </row>
-    <row r="466" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F466" s="5"/>
     </row>
-    <row r="467" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F467" s="5"/>
     </row>
-    <row r="468" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F468" s="5"/>
     </row>
-    <row r="469" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F469" s="5"/>
     </row>
-    <row r="470" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F470" s="5"/>
     </row>
-    <row r="471" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F471" s="5"/>
     </row>
-    <row r="472" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F472" s="5"/>
     </row>
-    <row r="473" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F473" s="5"/>
     </row>
-    <row r="474" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F474" s="5"/>
     </row>
-    <row r="475" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F475" s="5"/>
     </row>
-    <row r="476" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F476" s="5"/>
     </row>
-    <row r="477" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F477" s="5"/>
     </row>
-    <row r="478" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F478" s="5"/>
     </row>
-    <row r="479" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F479" s="5"/>
     </row>
-    <row r="480" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F480" s="5"/>
     </row>
-    <row r="481" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F481" s="5"/>
     </row>
-    <row r="482" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F482" s="5"/>
     </row>
-    <row r="483" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F483" s="5"/>
     </row>
-    <row r="484" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F484" s="5"/>
     </row>
-    <row r="485" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F485" s="5"/>
     </row>
-    <row r="486" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F486" s="5"/>
     </row>
-    <row r="487" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F487" s="5"/>
     </row>
-    <row r="488" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F488" s="5"/>
     </row>
-    <row r="489" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F489" s="5"/>
     </row>
-    <row r="490" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F490" s="5"/>
     </row>
-    <row r="491" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F491" s="5"/>
     </row>
-    <row r="492" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F492" s="5"/>
     </row>
-    <row r="493" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F493" s="5"/>
     </row>
-    <row r="494" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F494" s="5"/>
     </row>
-    <row r="495" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F495" s="5"/>
     </row>
-    <row r="496" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F496" s="5"/>
     </row>
-    <row r="497" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F497" s="5"/>
     </row>
-    <row r="498" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F498" s="5"/>
     </row>
-    <row r="499" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F499" s="5"/>
     </row>
-    <row r="500" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F500" s="5"/>
     </row>
-    <row r="501" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F501" s="5"/>
     </row>
   </sheetData>

</xml_diff>